<commit_message>
Bổ sung thời gian khách góp ý bài viết (lấy từ bình luận Google Docs) vào bảng tiến độ AIG
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D8MNR49cLoKAHjYy9hXWE4
</commit_message>
<xml_diff>
--- a/Kết quả công việc Agent Boss/Viec that - Tien do Content AIG/tien-do-content-aig-85-bai.xlsx
+++ b/Kết quả công việc Agent Boss/Viec that - Tien do Content AIG/tien-do-content-aig-85-bai.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Thời gian xử lý" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Tồn chờ khách AIG" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Chi tiết từng bài" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Góp ý bài viết" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Chi tiết từng bài'!$A$4:$N$64</definedName>
@@ -135,11 +136,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -985,7 +986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1055,15 +1056,15 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>KTS duyệt outline</t>
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>KTS duyệt outline (content gửi → KTS duyệt xong, gửi khách)</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="16" t="n">
         <v>2.6</v>
       </c>
       <c r="D5" s="4" t="n">
@@ -1075,27 +1076,27 @@
       <c r="F5" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="G5" s="16" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>Ngày content gửi → ngày gửi khách</t>
         </is>
       </c>
-      <c r="H5" s="16" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
         <is>
           <t>Bài "công ty cung cấp tinh bột sắn" mất 19 ngày do vướng trao đổi key → tính bằng thời gian trung bình các bài còn lại.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>KTS duyệt bài viết</t>
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Content gửi bài → KTS duyệt xong, gửi khách</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="16" t="n">
         <v>1.9</v>
       </c>
       <c r="D6" s="4" t="n">
@@ -1107,7 +1108,7 @@
       <c r="F6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="G6" s="16" t="inlineStr">
+      <c r="G6" s="15" t="inlineStr">
         <is>
           <t>Ngày content gửi bài → ngày gửi khách</t>
         </is>
@@ -1123,7 +1124,7 @@
       <c r="B7" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="16" t="n">
         <v>44.2</v>
       </c>
       <c r="D7" s="4" t="n">
@@ -1135,27 +1136,27 @@
       <c r="F7" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="G7" s="16" t="inlineStr">
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>Ngày gửi khách → ngày khách duyệt</t>
         </is>
       </c>
-      <c r="H7" s="16" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>14 outline khách đã duyệt nhưng sheet không ghi ngày duyệt nên không tính được.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Khách (AIG) duyệt bài viết</t>
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>KTS gửi bài → khách (AIG) duyệt</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="16" t="n">
         <v>28.1</v>
       </c>
       <c r="D8" s="4" t="n">
@@ -1172,22 +1173,22 @@
           <t>Ngày gửi khách → ngày đăng</t>
         </is>
       </c>
-      <c r="H8" s="16" t="inlineStr">
+      <c r="H8" s="15" t="inlineStr">
         <is>
           <t>Sheet không có ngày khách duyệt bài. AIG duyệt xong là đăng ngay, nên lấy ngày đăng làm mốc khách duyệt.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>Content viết bài (sau khi khách duyệt outline)</t>
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>Khách duyệt outline → content gửi bài cho KTS duyệt</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="16" t="n">
         <v>13</v>
       </c>
       <c r="D9" s="4" t="n">
@@ -1199,14 +1200,78 @@
       <c r="F9" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>Ngày khách duyệt outline → ngày content gửi bài</t>
         </is>
       </c>
-      <c r="H9" s="16" t="inlineStr">
+      <c r="H9" s="15" t="inlineStr">
         <is>
           <t>Bỏ 2 bài ghi ngày gửi bài (04/08) sớm hơn ngày khách duyệt outline (07/08) — ngày ghi bị lệch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>KTS gửi bài → khách góp ý, content bắt đầu sửa</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>12.1</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>Ngày gửi khách → ngày content trả lời góp ý đầu tiên của AIG trong file Docs</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Sheet không có cột ngày khách góp ý. Lấy từ lịch sử bình luận trong Google Docs: ngày content trả lời "đã điều chỉnh" ≈ ngày khách góp ý (khách góp ý trước đó hoặc cùng ngày).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>KTS gửi bài → content sửa xong góp ý cuối cùng</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>Ngày gửi khách → ngày content trả lời góp ý cuối cùng</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>Gồm cả các vòng khách góp ý lần 2, lần 3.</t>
         </is>
       </c>
     </row>
@@ -1290,7 +1355,7 @@
           <t>Outline</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>nguyên liệu đạt tiêu chuẩn xuất khẩu</t>
         </is>
@@ -1418,7 +1483,7 @@
           <t>Outline</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>nguyên liệu cho thực phẩm chức năng</t>
         </is>
@@ -1480,7 +1545,7 @@
           <t>Outline</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>công ty cung cấp nguyên liệu thực phẩm</t>
         </is>
@@ -1573,7 +1638,7 @@
           <t>Outline</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>giải pháp nguyên liệu cho doanh nghiệp</t>
         </is>
@@ -1604,7 +1669,7 @@
           <t>Outline</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>giải pháp nguyên liệu tùy chỉnh</t>
         </is>
@@ -1635,7 +1700,7 @@
           <t>Outline</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>nguyên liệu cho doanh nghiệp fmcg</t>
         </is>
@@ -1666,7 +1731,7 @@
           <t>Outline</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>giải pháp phát triển sản phẩm thực phẩm</t>
         </is>
@@ -1728,7 +1793,7 @@
           <t>Outline</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>nguyên liệu cho dược &amp; life science</t>
         </is>
@@ -2009,7 +2074,7 @@
           <t>Bài viết</t>
         </is>
       </c>
-      <c r="B28" s="16" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t>công ty cung cấp nước ép trái cây</t>
         </is>
@@ -2071,7 +2136,7 @@
           <t>Bài viết</t>
         </is>
       </c>
-      <c r="B30" s="16" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>công ty cung cấp tinh dầu thiên nhiên</t>
         </is>
@@ -2387,7 +2452,7 @@
           <t>Tối ưu</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -2425,7 +2490,7 @@
           <t>18</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>công ty chế biến trái cây đông lạnh</t>
         </is>
@@ -2489,7 +2554,7 @@
           <t>23</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>công ty cung cấp chất ổn định thực phẩm</t>
         </is>
@@ -2617,7 +2682,7 @@
           <t>40</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>công ty cung cấp nguyên liệu thực phẩm</t>
         </is>
@@ -2627,7 +2692,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -2675,7 +2740,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -2787,7 +2852,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>Bài viết đang chờ khách (AIG) duyệt</t>
         </is>
@@ -2851,7 +2916,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -2889,7 +2954,7 @@
           <t>71</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>giải pháp nguyên liệu cho doanh nghiệp</t>
         </is>
@@ -2899,7 +2964,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -2937,7 +3002,7 @@
           <t>72</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>giải pháp nguyên liệu tùy chỉnh</t>
         </is>
@@ -2947,7 +3012,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="D17" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -2985,7 +3050,7 @@
           <t>73</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>giải pháp phát triển sản phẩm thực phẩm</t>
         </is>
@@ -2995,7 +3060,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="D18" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -3043,7 +3108,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -3081,7 +3146,7 @@
           <t>77</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>nguyên liệu cho doanh nghiệp fmcg</t>
         </is>
@@ -3091,7 +3156,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D20" s="16" t="inlineStr">
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -3129,7 +3194,7 @@
           <t>78</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>nguyên liệu cho dược &amp; life science</t>
         </is>
@@ -3139,7 +3204,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr">
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -3251,7 +3316,7 @@
           <t>Tối ưu</t>
         </is>
       </c>
-      <c r="D23" s="16" t="inlineStr">
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -3289,7 +3354,7 @@
           <t>81</t>
         </is>
       </c>
-      <c r="B24" s="16" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>nguyên liệu đạt tiêu chuẩn xuất khẩu</t>
         </is>
@@ -3299,7 +3364,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D24" s="16" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -3343,7 +3408,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D25" s="16" t="inlineStr">
+      <c r="D25" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -3581,7 +3646,7 @@
           <t>94</t>
         </is>
       </c>
-      <c r="B29" s="16" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>nguyên liệu cho thực phẩm chức năng</t>
         </is>
@@ -3591,7 +3656,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D29" s="16" t="inlineStr">
+      <c r="D29" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -3765,7 +3830,7 @@
           <t>110</t>
         </is>
       </c>
-      <c r="B32" s="16" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
         <is>
           <t>nhà cung cấp nguyên liệu cho ngành sữa</t>
         </is>
@@ -3837,7 +3902,7 @@
           <t>111</t>
         </is>
       </c>
-      <c r="B33" s="16" t="inlineStr">
+      <c r="B33" s="15" t="inlineStr">
         <is>
           <t>nhà cung cấp nguyên liệu bánh kẹo</t>
         </is>
@@ -3909,7 +3974,7 @@
           <t>110</t>
         </is>
       </c>
-      <c r="B34" s="16" t="inlineStr">
+      <c r="B34" s="15" t="inlineStr">
         <is>
           <t>công ty cung cấp nước ép trái cây</t>
         </is>
@@ -3919,7 +3984,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D34" s="16" t="inlineStr">
+      <c r="D34" s="15" t="inlineStr">
         <is>
           <t>Bài viết đang chờ khách (AIG) duyệt</t>
         </is>
@@ -3987,7 +4052,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D35" s="16" t="inlineStr">
+      <c r="D35" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -4035,7 +4100,7 @@
           <t>Tối ưu</t>
         </is>
       </c>
-      <c r="D36" s="16" t="inlineStr">
+      <c r="D36" s="15" t="inlineStr">
         <is>
           <t>Bài viết đang chờ khách (AIG) duyệt</t>
         </is>
@@ -4093,7 +4158,7 @@
           <t>131</t>
         </is>
       </c>
-      <c r="B37" s="16" t="inlineStr">
+      <c r="B37" s="15" t="inlineStr">
         <is>
           <t>công ty cung cấp tinh dầu thiên nhiên</t>
         </is>
@@ -4103,7 +4168,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D37" s="16" t="inlineStr">
+      <c r="D37" s="15" t="inlineStr">
         <is>
           <t>Bài viết đang chờ khách (AIG) duyệt</t>
         </is>
@@ -4171,7 +4236,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D38" s="16" t="inlineStr">
+      <c r="D38" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -4219,7 +4284,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D39" s="16" t="inlineStr">
+      <c r="D39" s="15" t="inlineStr">
         <is>
           <t>Khách đã duyệt outline – content đang viết bài</t>
         </is>
@@ -4339,7 +4404,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D41" s="16" t="inlineStr">
+      <c r="D41" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -4387,7 +4452,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D42" s="16" t="inlineStr">
+      <c r="D42" s="15" t="inlineStr">
         <is>
           <t>Bài viết đang chờ khách (AIG) duyệt</t>
         </is>
@@ -4455,7 +4520,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D43" s="16" t="inlineStr">
+      <c r="D43" s="15" t="inlineStr">
         <is>
           <t>Bài viết đang chờ khách (AIG) duyệt</t>
         </is>
@@ -4659,7 +4724,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr">
+      <c r="D46" s="15" t="inlineStr">
         <is>
           <t>Khách đã duyệt outline – content đang viết bài</t>
         </is>
@@ -4707,7 +4772,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D47" s="16" t="inlineStr">
+      <c r="D47" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -4751,7 +4816,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D48" s="16" t="inlineStr">
+      <c r="D48" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -4847,7 +4912,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D50" s="16" t="inlineStr">
+      <c r="D50" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -4919,7 +4984,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D52" s="16" t="inlineStr">
+      <c r="D52" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ KTS duyệt / content đang sửa</t>
         </is>
@@ -4947,7 +5012,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D53" s="16" t="inlineStr">
+      <c r="D53" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ khách (AIG) duyệt</t>
         </is>
@@ -4987,7 +5052,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D54" s="16" t="inlineStr">
+      <c r="D54" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ KTS duyệt / content đang sửa</t>
         </is>
@@ -5023,7 +5088,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D55" s="16" t="inlineStr">
+      <c r="D55" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ KTS duyệt / content đang sửa</t>
         </is>
@@ -5051,7 +5116,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D56" s="16" t="inlineStr">
+      <c r="D56" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ KTS duyệt / content đang sửa</t>
         </is>
@@ -5079,7 +5144,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D57" s="16" t="inlineStr">
+      <c r="D57" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ KTS duyệt / content đang sửa</t>
         </is>
@@ -5115,7 +5180,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D58" s="16" t="inlineStr">
+      <c r="D58" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ KTS duyệt / content đang sửa</t>
         </is>
@@ -5151,7 +5216,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D59" s="16" t="inlineStr">
+      <c r="D59" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ KTS duyệt / content đang sửa</t>
         </is>
@@ -5187,7 +5252,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D60" s="16" t="inlineStr">
+      <c r="D60" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ KTS duyệt / content đang sửa</t>
         </is>
@@ -5215,7 +5280,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D61" s="16" t="inlineStr">
+      <c r="D61" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ KTS duyệt / content đang sửa</t>
         </is>
@@ -5271,7 +5336,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D63" s="16" t="inlineStr">
+      <c r="D63" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ KTS duyệt / content đang sửa</t>
         </is>
@@ -5299,7 +5364,7 @@
           <t>Viết mới</t>
         </is>
       </c>
-      <c r="D64" s="16" t="inlineStr">
+      <c r="D64" s="15" t="inlineStr">
         <is>
           <t>Outline đang chờ KTS duyệt / content đang sửa</t>
         </is>
@@ -5319,4 +5384,780 @@
   <autoFilter ref="A4:N64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Khách (AIG) góp ý bài viết – lấy từ bình luận trong Google Docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Người góp ý phía AIG: Kim Ngân, Đoàn Ly, Thảo Nguyễn, Business ASI, Thanh Phan. Người sửa phía SEONGON: Trân Lê, Lan Phương Vũ, Nhơn Hoài Lê.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Bài viết</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Ngày KTS gửi khách</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>AIG duyệt bài</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Số góp ý của AIG</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Ngày content bắt đầu sửa</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Số ngày (gửi → bắt đầu sửa)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Ngày sửa xong góp ý cuối</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Số ngày (gửi → sửa xong)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>bã sắn</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>25/06/2026</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>25/06/2026</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>07/07/2026</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>bột kem</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>25/06/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>25/06/2026</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>chế biến trái cây đông lạnh</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>20/07/2026</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>13/08/2026</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>nước dừa tươi</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>25/06/2026</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>25/06/2026</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>07/07/2026</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>thạch dừa</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>20/07/2026</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Yêu cầu duyệt</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>nguyên liệu cho ngành sữa</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>14/07/2026</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>pha chế đồ uống</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>sản xuất kẹo</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>16/07/2026</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>30/07/2026</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>nguyên liệu thực phẩm</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>16/07/2026</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>27/07/2026</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>kem không sữa</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>06/07/2026</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>16/07/2026</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>hương liệu</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>20/07/2026</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>12/08/2026</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>24/08/2026</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>NCC nguyên liệu ngành sữa</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>NCC nguyên liệu bánh kẹo</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>nước ép trái cây</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Yêu cầu duyệt</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>tinh bột sắn</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Đã sửa</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>15/09/2026</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>15/09/2026</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>tinh dầu thiên nhiên</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Đã sửa</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>nước dừa uht</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>trái cây đông lạnh</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>27/08/2026</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Yêu cầu duyệt</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr"/>
+      <c r="H22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>trái cây iqf</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>26/08/2026</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Yêu cầu duyệt</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>công nghệ uht</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>vảy ngũ cốc</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Duyệt</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>18/08/2026</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>